<commit_message>
Add NCT01797120 (PrE0102, PrECOG) to misc_studies: Layer 1-3 single-pass
Section 7 Study Parameters, doc pp.69-71, one main_soa table: 20 flat
activities, 71 marks (bbox check 71/71, independent re-check agrees),
19 annotations (a-o + *, ^, GBP symbol + pr1 source_note), 5 review
items D1-D5. Gate 0 FAIL; pipeline 0 errors; row audit 0
on-page-not-extracted. Manifest rows, stamped pages, review page,
collection + root indexes regenerated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YTf92PKd6z7Q2fy8dyrbbp
</commit_message>
<xml_diff>
--- a/collections/misc_studies/studies_protocols.xlsx
+++ b/collections/misc_studies/studies_protocols.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -479,6 +479,28 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NCT01797120</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PrECOG, LLC.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PrE0102</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Breast Cancer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -490,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -535,6 +557,23 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NCT01797120</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>69-71</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://ClinicalTrials.gov/ProvidedDocs/20/NCT01797120/Prot_000.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>